<commit_message>
Prepara execução em celular e atualiza situação da entrega
</commit_message>
<xml_diff>
--- a/android-native/docs/EasyVacc-Android-Testes.xlsx
+++ b/android-native/docs/EasyVacc-Android-Testes.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projeto" sheetId="1" r:id="Rf84f0cfa16f14d27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tecnicas" sheetId="2" r:id="Rc87f1a88c6644aff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="3" r:id="Rae72b0e8c28541f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execucoes" sheetId="4" r:id="R1390ccd229944e51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defeitos" sheetId="5" r:id="Rf2709664d4ae486a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documentacao" sheetId="6" r:id="R803bfa4cb9a74511"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemplo" sheetId="7" r:id="Rd8980bf097cb450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projeto" sheetId="1" r:id="R06268709d45a4624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tecnicas" sheetId="2" r:id="R9806aff58a734d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="3" r:id="R470cba2d963d4405"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execucoes" sheetId="4" r:id="R7bc9b038dcdf4503"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defeitos" sheetId="5" r:id="R2be0cda1d9954534"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documentacao" sheetId="6" r:id="R175053af2e89484b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemplo" sheetId="7" r:id="Rac944f95a1df48b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2342,7 +2342,7 @@
         <x:v>Verificação do artefato, sem instalar ou executar o APK em Android.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="66" hidden="0" customHeight="1">
+    <x:row r="8" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A8" s="8" t="str">
         <x:v>EXN03</x:v>
       </x:c>
@@ -2362,7 +2362,7 @@
         <x:v>2.0.0; 3ec6a339981c24ac…; commit 27d4167</x:v>
       </x:c>
       <x:c r="G8" s="8" t="str">
-        <x:v>Não foi possível executar o fluxo completo: adb falhou ao criar sua pasta de credenciais.</x:v>
+        <x:v>Execução em Android ainda pendente. Acesso adb recuperado, mas nenhum aparelho conectado na última consulta.</x:v>
       </x:c>
       <x:c r="H8" s="8" t="str">
         <x:v>Bloqueado</x:v>
@@ -2372,7 +2372,7 @@
       </x:c>
       <x:c r="J8" s="8" t="str"/>
       <x:c r="K8" s="8" t="str">
-        <x:v>CTN01-CTN16 permanecem planejados para teste manual. Runner de banco e abertura da tela apenas compilado.</x:v>
+        <x:v>CTN01-CTN16 aguardam teste manual. Runner Android compilado. test-device.ps1 automatiza instalação, execução e registro de evidência.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="65" customHeight="1">
@@ -2964,7 +2964,7 @@
         <x:v>ID da reexecução</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="66" hidden="0" customHeight="1">
+    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A5" s="8" t="str">
         <x:v>DFN01</x:v>
       </x:c>
@@ -2993,7 +2993,7 @@
         <x:v>Pedro Marcos Quintanilha de Oliveira Nunes</x:v>
       </x:c>
       <x:c r="J5" s="8" t="str">
-        <x:v>Commit local 158fbcf; ShareFlow.preview valida e preserva o texto.</x:v>
+        <x:v>Commit 27d4167. ShareFlow.preview valida e preserva o texto.</x:v>
       </x:c>
       <x:c r="K5" s="8" t="str">
         <x:v>EXN01; validação JVM, Android ainda pendente.</x:v>
@@ -3684,7 +3684,7 @@
         <x:v>Histórico GitHub</x:v>
       </x:c>
       <x:c r="B15" s="8" t="str">
-        <x:v>Repositório histórico: https://github.com/kawanzn/sistema_de_vacina2 . Novo código no commit 27d4167; não foi enviado. A entrega atual está nos arquivos APK, ZIP de fontes e nesta planilha.</x:v>
+        <x:v>Código, APK e planilha publicados em https://github.com/kawanzn/sistema_de_vacina2 . Código nativo: commit 27d4167. Instalador: releases/EasyVacc-Android-2.0.0.apk.</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
         <x:v>Commits e links que demonstram a evolução.</x:v>

</xml_diff>